<commit_message>
formatting edit for prep method
</commit_message>
<xml_diff>
--- a/template/sgp_context_template.xlsx
+++ b/template/sgp_context_template.xlsx
@@ -5,18 +5,18 @@
   <workbookPr showInkAnnotation="0" autoCompressPictures="0"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/unafarrell/Dropbox/Database/Templates/git/sgp-context-template/templates/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/unafarrell/Dropbox/Database/Templates/git/sgp-context-template/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{AE734616-9679-5C49-885D-1E9D2721BDDD}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{CE7D8650-6E97-3A45-BE22-36488B5F0B1D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4940" yWindow="600" windowWidth="32760" windowHeight="18640" tabRatio="500" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="4940" yWindow="600" windowWidth="32760" windowHeight="18640" tabRatio="500" activeTab="3" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Metadata + Guide" sheetId="8" r:id="rId1"/>
     <sheet name="Sites" sheetId="3" r:id="rId2"/>
     <sheet name="Samples" sheetId="2" r:id="rId3"/>
-    <sheet name="PrepMethods" sheetId="10" r:id="rId4"/>
+    <sheet name="Prep Method" sheetId="10" r:id="rId4"/>
     <sheet name="Dictionary of Sed Structures" sheetId="9" r:id="rId5"/>
     <sheet name="Dropdowns" sheetId="7" state="hidden" r:id="rId6"/>
   </sheets>
@@ -2225,7 +2225,7 @@
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="62">
+  <cellXfs count="61">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
@@ -2312,6 +2312,28 @@
     <xf numFmtId="0" fontId="0" fillId="6" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="left" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
+    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="201" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
@@ -2325,31 +2347,6 @@
       <alignment horizontal="left"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="8" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="10" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="10" borderId="0" xfId="0" applyFill="1"/>
-    <xf numFmtId="0" fontId="5" fillId="8" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="13" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="164" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="14" fontId="14" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="left"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="201" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
   </cellXfs>
@@ -2943,69 +2940,68 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:4" s="42" customFormat="1" ht="69" customHeight="1">
-      <c r="A1" s="56" t="s">
+      <c r="A1" s="50" t="s">
         <v>507</v>
       </c>
-      <c r="B1" s="56"/>
+      <c r="B1" s="50"/>
     </row>
     <row r="2" spans="1:4" s="42" customFormat="1" ht="15" customHeight="1">
-      <c r="A2" s="57" t="s">
+      <c r="A2" s="51" t="s">
         <v>493</v>
       </c>
-      <c r="B2" s="58">
+      <c r="B2" s="52">
         <v>2</v>
       </c>
     </row>
     <row r="3" spans="1:4" s="42" customFormat="1" ht="15" customHeight="1">
-      <c r="A3" s="57" t="s">
+      <c r="A3" s="51" t="s">
         <v>494</v>
       </c>
-      <c r="B3" s="59">
+      <c r="B3" s="53">
         <v>46296</v>
       </c>
     </row>
     <row r="4" spans="1:4" s="6" customFormat="1" ht="15" customHeight="1">
-      <c r="A4" s="57" t="s">
+      <c r="A4" s="51" t="s">
         <v>495</v>
       </c>
-      <c r="B4" s="60" t="s">
+      <c r="B4" s="54" t="s">
         <v>498</v>
       </c>
-      <c r="C4" s="53"/>
     </row>
     <row r="5" spans="1:4" s="6" customFormat="1" ht="15" customHeight="1">
-      <c r="A5" s="57" t="s">
+      <c r="A5" s="51" t="s">
         <v>496</v>
       </c>
-      <c r="B5" s="60" t="s">
+      <c r="B5" s="54" t="s">
         <v>500</v>
       </c>
     </row>
     <row r="6" spans="1:4" s="6" customFormat="1" ht="15" customHeight="1">
-      <c r="A6" s="57" t="s">
+      <c r="A6" s="51" t="s">
         <v>497</v>
       </c>
-      <c r="B6" s="61" t="s">
+      <c r="B6" s="55" t="s">
         <v>499</v>
       </c>
     </row>
     <row r="7" spans="1:4" s="8" customFormat="1" ht="175" customHeight="1">
-      <c r="A7" s="48" t="s">
+      <c r="A7" s="56" t="s">
         <v>513</v>
       </c>
-      <c r="B7" s="48"/>
+      <c r="B7" s="56"/>
       <c r="C7" s="26"/>
       <c r="D7" s="26"/>
     </row>
     <row r="8" spans="1:4" s="6" customFormat="1" ht="15" customHeight="1">
-      <c r="A8" s="57"/>
-      <c r="B8" s="60"/>
+      <c r="A8" s="51"/>
+      <c r="B8" s="54"/>
     </row>
     <row r="9" spans="1:4" ht="51" customHeight="1">
-      <c r="A9" s="54" t="s">
+      <c r="A9" s="48" t="s">
         <v>501</v>
       </c>
-      <c r="B9" s="55"/>
+      <c r="B9" s="49"/>
     </row>
     <row r="10" spans="1:4" ht="19">
       <c r="A10" s="44" t="s">
@@ -3032,10 +3028,10 @@
       <c r="B14" s="43"/>
     </row>
     <row r="15" spans="1:4" s="8" customFormat="1" ht="217" customHeight="1">
-      <c r="A15" s="48" t="s">
+      <c r="A15" s="56" t="s">
         <v>511</v>
       </c>
-      <c r="B15" s="48"/>
+      <c r="B15" s="56"/>
       <c r="C15" s="26"/>
       <c r="D15" s="26"/>
     </row>
@@ -3534,10 +3530,10 @@
       <c r="R1" s="38"/>
       <c r="S1" s="38"/>
       <c r="T1" s="38"/>
-      <c r="U1" s="49" t="s">
+      <c r="U1" s="57" t="s">
         <v>133</v>
       </c>
-      <c r="V1" s="49"/>
+      <c r="V1" s="57"/>
       <c r="W1" s="24"/>
       <c r="X1" s="24"/>
       <c r="Y1" s="25"/>
@@ -4201,22 +4197,22 @@
   </cols>
   <sheetData>
     <row r="1" spans="1:25">
-      <c r="A1" s="50" t="s">
+      <c r="A1" s="58" t="s">
         <v>225</v>
       </c>
-      <c r="B1" s="50"/>
-      <c r="C1" s="50"/>
-      <c r="D1" s="50"/>
+      <c r="B1" s="58"/>
+      <c r="C1" s="58"/>
+      <c r="D1" s="58"/>
       <c r="E1" s="14" t="s">
         <v>226</v>
       </c>
       <c r="F1" s="14"/>
       <c r="G1" s="14"/>
-      <c r="H1" s="51" t="s">
+      <c r="H1" s="59" t="s">
         <v>227</v>
       </c>
-      <c r="I1" s="51"/>
-      <c r="J1" s="51"/>
+      <c r="I1" s="59"/>
+      <c r="J1" s="59"/>
       <c r="K1" s="5" t="s">
         <v>228</v>
       </c>
@@ -4224,18 +4220,18 @@
       <c r="M1" s="19" t="s">
         <v>109</v>
       </c>
-      <c r="N1" s="52" t="s">
+      <c r="N1" s="60" t="s">
         <v>260</v>
       </c>
-      <c r="O1" s="52"/>
-      <c r="P1" s="52"/>
-      <c r="Q1" s="52"/>
-      <c r="R1" s="52"/>
-      <c r="S1" s="50" t="s">
+      <c r="O1" s="60"/>
+      <c r="P1" s="60"/>
+      <c r="Q1" s="60"/>
+      <c r="R1" s="60"/>
+      <c r="S1" s="58" t="s">
         <v>142</v>
       </c>
-      <c r="T1" s="50"/>
-      <c r="U1" s="50"/>
+      <c r="T1" s="58"/>
+      <c r="U1" s="58"/>
       <c r="V1" s="19" t="s">
         <v>237</v>
       </c>

</xml_diff>